<commit_message>
Update group count (L3 EM, M2 IEAP)
</commit_message>
<xml_diff>
--- a/data/L3-EM.xlsx
+++ b/data/L3-EM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivier/SSDS/enseignement/UFR STAPS/Direction/Outils/celcatreport/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olivier/SSDS/direction/Outils/celcatreport/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{829429A6-2171-D447-AD1A-8F9337E05CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02E7CE04-1C51-2E4B-9900-7ED0D8F71F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19580" xr2:uid="{154AE90F-D41B-8B49-BA91-D855BEB6F170}"/>
   </bookViews>
@@ -585,7 +585,7 @@
         <v>26</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -617,7 +617,7 @@
         <v>28</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -655,7 +655,7 @@
         <v>66</v>
       </c>
       <c r="J4">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>12</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -745,7 +745,7 @@
         <v>6</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -777,7 +777,7 @@
         <v>12</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -809,7 +809,7 @@
         <v>18</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -841,7 +841,7 @@
         <v>12</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -873,7 +873,7 @@
         <v>20</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -905,7 +905,7 @@
         <v>12</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -937,7 +937,7 @@
         <v>16</v>
       </c>
       <c r="H13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -969,7 +969,7 @@
         <v>10</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1001,13 +1001,13 @@
         <v>26</v>
       </c>
       <c r="H15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I15">
         <v>10</v>
       </c>
       <c r="J15">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>